<commit_message>
Programas y proyectos: actas y resoluciones por programa o proyecto
Las actas se registran por programa o proyecto, no en general:

- Hoja Programas, y columna «Programa o proyecto» (varios, con punto y
  coma; vacío = asunto general) en Actas y Resoluciones. La resolución
  hereda los de su acta salvo que diga otros.
- La página los muestra como etiquetas, con filtro en Actas y Resoluciones,
  tarjeta en el panel y búsqueda. Un acta pertenece a un programa si ella
  o alguna de sus resoluciones lo nombra.
- Cada grupo de acceso recibe solo los programas que usa. Un Excel sin la
  hoja ni las columnas se publica igual.
- La documentación explica la contraseña del Excel y las frases en
  palabras simples.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FkuX6y6rjtHhRzfZ7rBQRg
</commit_message>
<xml_diff>
--- a/plantilla/Quorum_matriz.xlsx
+++ b/plantilla/Quorum_matriz.xlsx
@@ -9,11 +9,12 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuerpos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actas" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resoluciones" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Normativa" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cambios" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="7" state="hidden" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Programas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actas" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resoluciones" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Normativa" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cambios" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="8" state="hidden" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -206,37 +207,17 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>La sigla de la hoja Cuerpos.</t>
+        <t>Sin repetirse. Es como se escribe en las hojas Actas y Resoluciones.</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>dd/mm/aaaa. Con el cuerpo, es lo que identifica al acta.</t>
+        <t>Programa o Proyecto.</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Ordinaria o Extraordinaria.</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t>Opcional. Solo si la sesión tiene número.</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t>Enlace al PDF en la carpeta. Opcional.</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <t>Enlace al PDF firmado. Mientras esté vacío, el acta se muestra como provisional.</t>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <t>Cuándo se aprobó el acta definitiva (normalmente, en la sesión siguiente).</t>
+        <t>FIAS, FAP o FEIG.</t>
       </text>
     </comment>
   </commentList>
@@ -256,27 +237,37 @@
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>La del acta donde se resolvió.</t>
+        <t>dd/mm/aaaa. Con el cuerpo, es lo que identifica al acta.</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>El número del punto: 3, no «tercero». Cuerpo + fecha + punto identifican a la resolución.</t>
+        <t>Ordinaria o Extraordinaria.</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>El texto o un resumen fiel de lo resuelto.</t>
+        <t>Opcional. Solo si la sesión tiene número.</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Para filtrar. Se puede escribir otra si ninguna sirve.</t>
+        <t>De cuál trata la sesión (como está en la hoja Programas). Si trata de varios, sepáralos con punto y coma. Vacío = asunto general.</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Si la resolución tiene documento propio (certificación, extracto).</t>
+        <t>Enlace al PDF en la carpeta. Opcional.</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>Enlace al PDF firmado. Mientras esté vacío, el acta se muestra como provisional.</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>Cuándo se aprobó el acta definitiva (normalmente, en la sesión siguiente).</t>
       </text>
     </comment>
   </commentList>
@@ -291,42 +282,37 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Sin repetirse. Es como se la nombra en la hoja Cambios.</t>
+        <t>La sigla de la hoja Cuerpos.</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Reglamento, Manual, Política…</t>
+        <t>La del acta donde se resolvió.</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>FIAS, FAP o FEIG.</t>
+        <t>El número del punto: 3, no «tercero». Cuerpo + fecha + punto identifican a la resolución.</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Sigla del cuerpo competente (p. ej. el Manual de Ciclo lo aprueba la JA-FAP).</t>
+        <t>El texto o un resumen fiel de lo resuelto.</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Fecha de la sesión que la aprobó.</t>
+        <t>Para filtrar. Se puede escribir otra si ninguna sirve.</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Opcional. Con órgano + fecha + punto, la norma queda enlazada a su resolución.</t>
+        <t>Por omisión, la resolución es del programa o proyecto de su acta. Escríbelo aquí solo si esta resolución trata de otro, o de uno solo entre varios. Varios: separados con punto y coma.</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>PDF del texto aprobado.</t>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
-      <text>
-        <t>Opcional. Vacío = el mismo grupo del órgano que la aprueba.</t>
+        <t>Si la resolución tiene documento propio (certificación, extracto).</t>
       </text>
     </comment>
   </commentList>
@@ -334,6 +320,56 @@
 </file>
 
 <file path=xl/comments/comment5.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Quórum</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Sin repetirse. Es como se la nombra en la hoja Cambios.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Reglamento, Manual, Política…</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>FIAS, FAP o FEIG.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Sigla del cuerpo competente (p. ej. el Manual de Ciclo lo aprueba la JA-FAP).</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Fecha de la sesión que la aprobó.</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Opcional. Con órgano + fecha + punto, la norma queda enlazada a su resolución.</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>PDF del texto aprobado.</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>Opcional. Vacío = el mismo grupo del órgano que la aprueba.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment6.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Quórum</author>
@@ -398,40 +434,55 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tActas" displayName="tActas" ref="A1:H2" headerRowCount="1">
-  <autoFilter ref="A1:H2"/>
-  <tableColumns count="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tProgramas" displayName="tProgramas" ref="A1:D2" headerRowCount="1">
+  <autoFilter ref="A1:D2"/>
+  <tableColumns count="4">
+    <tableColumn id="1" name="Programa o proyecto"/>
+    <tableColumn id="2" name="Tipo"/>
+    <tableColumn id="3" name="Entidad"/>
+    <tableColumn id="4" name="Observaciones"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tActas" displayName="tActas" ref="A1:I2" headerRowCount="1">
+  <autoFilter ref="A1:I2"/>
+  <tableColumns count="9">
     <tableColumn id="1" name="Cuerpo colegiado"/>
     <tableColumn id="2" name="Fecha de la sesión"/>
     <tableColumn id="3" name="Tipo de sesión"/>
     <tableColumn id="4" name="N.º de sesión"/>
-    <tableColumn id="5" name="Acta provisional (enlace)"/>
-    <tableColumn id="6" name="Acta definitiva (enlace)"/>
-    <tableColumn id="7" name="Fecha de aprobación del acta definitiva"/>
-    <tableColumn id="8" name="Observaciones"/>
+    <tableColumn id="5" name="Programa o proyecto"/>
+    <tableColumn id="6" name="Acta provisional (enlace)"/>
+    <tableColumn id="7" name="Acta definitiva (enlace)"/>
+    <tableColumn id="8" name="Fecha de aprobación del acta definitiva"/>
+    <tableColumn id="9" name="Observaciones"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
 </table>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tResoluciones" displayName="tResoluciones" ref="A1:G2" headerRowCount="1">
-  <autoFilter ref="A1:G2"/>
-  <tableColumns count="7">
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tResoluciones" displayName="tResoluciones" ref="A1:H2" headerRowCount="1">
+  <autoFilter ref="A1:H2"/>
+  <tableColumns count="8">
     <tableColumn id="1" name="Cuerpo colegiado"/>
     <tableColumn id="2" name="Fecha de la sesión"/>
     <tableColumn id="3" name="Punto del orden del día"/>
     <tableColumn id="4" name="Lo que se resolvió"/>
     <tableColumn id="5" name="Materia"/>
-    <tableColumn id="6" name="Enlace (opcional)"/>
-    <tableColumn id="7" name="Observaciones"/>
+    <tableColumn id="6" name="Programa o proyecto (solo si es distinto del acta)"/>
+    <tableColumn id="7" name="Enlace (opcional)"/>
+    <tableColumn id="8" name="Observaciones"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
 </table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tNormativa" displayName="tNormativa" ref="A1:I2" headerRowCount="1">
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="tNormativa" displayName="tNormativa" ref="A1:I2" headerRowCount="1">
   <autoFilter ref="A1:I2"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Nombre de la norma"/>
@@ -448,8 +499,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="tCambios" displayName="tCambios" ref="A1:L2" headerRowCount="1">
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="tCambios" displayName="tCambios" ref="A1:L2" headerRowCount="1">
   <autoFilter ref="A1:L2"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Norma afectada"/>
@@ -758,7 +809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -795,117 +846,124 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2. Actas: un renglón por sesión. Cuerpo + fecha de la sesión identifican al acta. Mientras no tenga enlace al acta definitiva ni fecha de aprobación, se muestra como provisional.</t>
+          <t>2. Programas: un renglón por cada programa o proyecto. Con ellos se llena la columna «Programa o proyecto» de Actas y Resoluciones, y así se puede consultar todo lo de un proyecto junto. Si algo es general (no es de ningún proyecto), esa columna se deja vacía.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>3. Resoluciones: un renglón por cada punto en que se resolvió algo. Cuerpo + fecha + punto la identifican: «en la Junta Administrativa del 8 de agosto de 2026, en el tercer punto» se escribe JA-FAP · 08/08/2026 · 3.</t>
+          <t>3. Actas: un renglón por sesión. Cuerpo + fecha de la sesión identifican al acta. Si la sesión trata de uno o varios programas o proyectos, se escriben en «Programa o proyecto», separados con punto y coma. Mientras no tenga enlace al acta definitiva ni fecha de aprobación, se muestra como provisional.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>4. Normativa: un renglón por norma, con el órgano que la aprueba y la fecha (y si se sabe, el punto) en que se aprobó.</t>
+          <t>4. Resoluciones: un renglón por cada punto en que se resolvió algo. Cuerpo + fecha + punto la identifican: «en la Junta Administrativa del 8 de agosto de 2026, en el tercer punto» se escribe JA-FAP · 08/08/2026 · 3. Por omisión es del programa o proyecto de su acta; la columna de programa solo se llena si trata de otro.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>5. Cambios: un renglón cada vez que una resolución reforma, codifica, deroga, deja sin efecto o aclara una norma u otra resolución.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+          <t>5. Normativa: un renglón por norma, con el órgano que la aprueba y la fecha (y si se sabe, el punto) en que se aprobó.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>6. Cambios: un renglón cada vez que una resolución reforma, codifica, deroga, deja sin efecto o aclara una norma u otra resolución.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>La vigencia no se escribe: se deduce</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>No hay columna «vigente». Quórum la calcula de la hoja Cambios, a la fecha que se pregunte: una norma con una Derogación es derogada desde esa fecha; con una Reforma o Codificación, sigue vigente con texto nuevo.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Cuando un acta nueva da de baja algo, solo se añade un renglón en Cambios. El renglón viejo no se toca: así nunca hay dos lugares que se contradigan.</t>
+          <t>No hay columna «vigente». Quórum la calcula de la hoja Cambios, a la fecha que se pregunte: una norma con una Derogación es derogada desde esa fecha; con una Reforma o Codificación, sigue vigente con texto nuevo.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>Cuando un acta nueva da de baja algo, solo se añade un renglón en Cambios. El renglón viejo no se toca: así nunca hay dos lugares que se contradigan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t>Si el cambio rige desde otra fecha (p. ej. «a partir del 1 de enero»), va en «Rige desde». Hasta entonces, Quórum lo muestra como cambio próximo.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Ejemplo de un renglón en Cambios</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Norma afectada: Manual Operativo del Ciclo de Proyectos del FAP · Tipo de cambio: Reforma · Resuelto por: JA-FAP · 08/08/2026 · 3 · Texto vigente: enlace al manual reformado.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Confidencialidad: tres reglas</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>1. Este libro se protege con contraseña: Archivo → Información → Proteger libro → Cifrar con contraseña. El robot lo abre con esa contraseña, guardada como secreto en GitHub; sin ella, el enlace de descarga solo entrega un archivo cerrado.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2. Los enlaces a los PDF deben ser de la carpeta compartida solo con quien corresponde, nunca «cualquier persona con el vínculo».</t>
+          <t>1. Este libro se protege con contraseña, como un PDF: en Excel de escritorio, Archivo → Información → Proteger libro → Cifrar con contraseña. Es una contraseña que tú inventas y que se guarda en GitHub como secreto (EXCEL_CLAVE): con ella el robot abre el libro. Sin ella, el enlace de descarga solo entrega un archivo cerrado. Este libro se edita en Excel de escritorio (Excel en el navegador no abre libros con contraseña).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
+          <t>2. Los enlaces a los PDF deben ser de la carpeta compartida solo con quien corresponde, nunca «cualquier persona con el vínculo».</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
           <t>3. No se cambia el nombre de las hojas ni de los encabezados de la fila 1. Las columnas sí se pueden reordenar o ensanchar.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>Publicar</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>El robot revisa este libro todos los días y publica lo que encuentre. Para publicar en el momento: en GitHub, pestaña Actions → «Publicar Quórum» → Run workflow.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>El robot revisa este libro todos los días y publica lo que encuentre. Para publicar en el momento: en GitHub, pestaña Actions → «Publicar Quórum» → Run workflow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>Si algo no cuadra (una resolución sin su acta, un cambio que apunta a una norma que no existe), Quórum lo muestra en «Revisión de la matriz», con la hoja y el renglón.</t>
         </is>
@@ -1048,7 +1106,65 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="46" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Programa o proyecto</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Entidad</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Observaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="B2:B2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor de la lista" error="Elige un valor de la lista. Si es un cuerpo o una norma nueva, añádelo primero en su hoja." type="list">
+      <formula1>Listas!$C$2:$C$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor de la lista" error="Elige un valor de la lista. Si es un cuerpo o una norma nueva, añádelo primero en su hoja." type="list">
+      <formula1>Listas!$A$2:$A$4</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1057,8 +1173,9 @@
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="34" customWidth="1" min="5" max="5"/>
     <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="46" customHeight="1">
@@ -1084,20 +1201,25 @@
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
+          <t>Programa o proyecto</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
           <t>Acta provisional (enlace)</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Acta definitiva (enlace)</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>Fecha de aprobación del acta definitiva</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -1105,8 +1227,8 @@
     </row>
     <row r="2">
       <c r="B2" s="5" t="n"/>
-      <c r="G2" s="5" t="n"/>
-      <c r="H2" s="2" t="n"/>
+      <c r="H2" s="5" t="n"/>
+      <c r="I2" s="2" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="4">
@@ -1119,7 +1241,7 @@
     <dataValidation sqref="C2:C2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor de la lista" error="Elige un valor de la lista. Si es un cuerpo o una norma nueva, añádelo primero en su hoja." type="list">
       <formula1>Listas!$B$2:$B$3</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fecha" error="Escribe una fecha: dd/mm/aaaa." type="date" operator="greaterThan">
+    <dataValidation sqref="H2:H2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fecha" error="Escribe una fecha: dd/mm/aaaa." type="date" operator="greaterThan">
       <formula1>DATE(1990,1,1)</formula1>
     </dataValidation>
   </dataValidations>
@@ -1131,13 +1253,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1145,8 +1267,9 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="46" customHeight="1">
@@ -1177,10 +1300,15 @@
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
+          <t>Programa o proyecto (solo si es distinto del acta)</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
           <t>Enlace (opcional)</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -1189,7 +1317,7 @@
     <row r="2">
       <c r="B2" s="5" t="n"/>
       <c r="D2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="3">
@@ -1200,7 +1328,7 @@
       <formula1>DATE(1990,1,1)</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor de la lista" error="Elige un valor de la lista. Si es un cuerpo o una norma nueva, añádelo primero en su hoja." type="list">
-      <formula1>Listas!$D$2:$D$11</formula1>
+      <formula1>Listas!$E$2:$E$11</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1211,7 +1339,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1286,7 +1414,7 @@
   </sheetData>
   <dataValidations count="4">
     <dataValidation sqref="B2:B2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor de la lista" error="Elige un valor de la lista. Si es un cuerpo o una norma nueva, añádelo primero en su hoja." type="list">
-      <formula1>Listas!$C$2:$C$10</formula1>
+      <formula1>Listas!$D$2:$D$10</formula1>
     </dataValidation>
     <dataValidation sqref="C2:C2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor de la lista" error="Elige un valor de la lista. Si es un cuerpo o una norma nueva, añádelo primero en su hoja." type="list">
       <formula1>Listas!$A$2:$A$4</formula1>
@@ -1306,7 +1434,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1409,7 +1537,7 @@
       <formula1>DATE(1990,1,1)</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor de la lista" error="Elige un valor de la lista. Si es un cuerpo o una norma nueva, añádelo primero en su hoja." type="list">
-      <formula1>Listas!$E$2:$E$7</formula1>
+      <formula1>Listas!$F$2:$F$7</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor de la lista" error="Elige un valor de la lista. Si es un cuerpo o una norma nueva, añádelo primero en su hoja." type="list">
       <formula1>Cuerpos!$A$2:$A$2000</formula1>
@@ -1429,13 +1557,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1443,6 +1571,7 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1458,15 +1587,20 @@
       </c>
       <c r="C1" s="6" t="inlineStr">
         <is>
+          <t>TIPOS_PROG</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
           <t>TIPOS_NORMA</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>MATERIAS</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>TIPOS_CAMBIO</t>
         </is>
@@ -1485,15 +1619,20 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>Estatuto</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Normativa</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Reforma</t>
         </is>
@@ -1512,15 +1651,20 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>Proyecto</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>Reglamento</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Presupuesto y finanzas</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Reforma parcial</t>
         </is>
@@ -1532,111 +1676,111 @@
           <t>FEIG</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Manual</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Inversiones</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Codificación</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Política</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Proyectos y convocatorias</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Derogación</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Procedimiento</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Convenios y alianzas</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Deja sin efecto</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Instructivo</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Talento humano</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Aclaración</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Lineamiento</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>Designaciones</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Código</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>Gobierno corporativo</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>Otro</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>Administrativo</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>Otros</t>
         </is>

</xml_diff>